<commit_message>
提交在IX9（Intel Xeon CPU Max 9462）上跑的结果
</commit_message>
<xml_diff>
--- a/doc/GEMM微内核的选择.xlsx
+++ b/doc/GEMM微内核的选择.xlsx
@@ -200,22 +200,22 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -1158,7 +1158,7 @@
     <col min="6" max="6" width="9.66666666666667" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5">
+    <row r="1" spans="1:6">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1203,20 +1203,20 @@
       <c r="B4">
         <v>4</v>
       </c>
-      <c r="C4" s="5">
-        <f>A4</f>
+      <c r="C4" s="7">
+        <f t="shared" ref="C4:C9" si="0">A4</f>
         <v>1</v>
       </c>
-      <c r="D4" s="5">
-        <f>CEILING(B4/4,1)</f>
+      <c r="D4" s="7">
+        <f t="shared" ref="D4:D9" si="1">CEILING(B4/4,1)</f>
         <v>1</v>
       </c>
-      <c r="E4" s="5">
-        <f>C4*D4</f>
+      <c r="E4" s="7">
+        <f t="shared" ref="E4:E9" si="2">C4*D4</f>
         <v>1</v>
       </c>
-      <c r="F4" s="5">
-        <f>SUM(C4:E4)</f>
+      <c r="F4" s="7">
+        <f t="shared" ref="F4:F9" si="3">SUM(C4:E4)</f>
         <v>3</v>
       </c>
     </row>
@@ -1227,44 +1227,44 @@
       <c r="B5">
         <v>8</v>
       </c>
-      <c r="C5" s="5">
-        <f>A5</f>
+      <c r="C5" s="7">
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
-      <c r="D5" s="5">
-        <f>CEILING(B5/4,1)</f>
+      <c r="D5" s="7">
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="E5" s="5">
-        <f>C5*D5</f>
+      <c r="E5" s="7">
+        <f t="shared" si="2"/>
         <v>2</v>
       </c>
-      <c r="F5" s="5">
-        <f>SUM(C5:E5)</f>
+      <c r="F5" s="7">
+        <f t="shared" si="3"/>
         <v>5</v>
       </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="5">
-        <v>4</v>
-      </c>
-      <c r="B6" s="5">
-        <v>4</v>
-      </c>
-      <c r="C6" s="5">
-        <f>A6</f>
-        <v>4</v>
-      </c>
-      <c r="D6" s="5">
-        <f>CEILING(B6/4,1)</f>
+      <c r="A6" s="7">
+        <v>4</v>
+      </c>
+      <c r="B6" s="7">
+        <v>4</v>
+      </c>
+      <c r="C6" s="7">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="D6" s="7">
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="E6" s="5">
-        <f>C6*D6</f>
-        <v>4</v>
-      </c>
-      <c r="F6" s="5">
-        <f>SUM(C6:E6)</f>
+      <c r="E6" s="7">
+        <f t="shared" si="2"/>
+        <v>4</v>
+      </c>
+      <c r="F6" s="7">
+        <f t="shared" si="3"/>
         <v>9</v>
       </c>
     </row>
@@ -1276,19 +1276,19 @@
         <v>8</v>
       </c>
       <c r="C7" s="4">
-        <f>A7</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="D7" s="4">
-        <f>CEILING(B7/4,1)</f>
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
       <c r="E7" s="4">
-        <f>C7*D7</f>
+        <f t="shared" si="2"/>
         <v>8</v>
       </c>
       <c r="F7" s="4">
-        <f>SUM(C7:E7)</f>
+        <f t="shared" si="3"/>
         <v>14</v>
       </c>
     </row>
@@ -1300,43 +1300,43 @@
         <v>8</v>
       </c>
       <c r="C8">
-        <f>A8</f>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
       <c r="D8">
-        <f>CEILING(B8/4,1)</f>
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
       <c r="E8">
-        <f>C8*D8</f>
+        <f t="shared" si="2"/>
         <v>10</v>
       </c>
       <c r="F8">
-        <f>SUM(C8:E8)</f>
+        <f t="shared" si="3"/>
         <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="5">
-        <v>4</v>
-      </c>
-      <c r="B9" s="5">
+      <c r="A9" s="7">
+        <v>4</v>
+      </c>
+      <c r="B9" s="7">
         <v>12</v>
       </c>
-      <c r="C9" s="5">
-        <f>A9</f>
-        <v>4</v>
-      </c>
-      <c r="D9" s="5">
-        <f>CEILING(B9/4,1)</f>
+      <c r="C9" s="7">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="D9" s="7">
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="E9" s="5">
-        <f>C9*D9</f>
+      <c r="E9" s="7">
+        <f t="shared" si="2"/>
         <v>12</v>
       </c>
-      <c r="F9" s="5">
-        <f>SUM(C9:E9)</f>
+      <c r="F9" s="7">
+        <f t="shared" si="3"/>
         <v>19</v>
       </c>
     </row>
@@ -1360,7 +1360,7 @@
     <col min="1" max="5" width="6.66666666666667" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:5">
+    <row r="1" spans="1:6">
       <c r="B1" s="1" t="s">
         <v>8</v>
       </c>
@@ -1406,19 +1406,19 @@
         <v>8</v>
       </c>
       <c r="C4">
-        <f>A4</f>
+        <f t="shared" ref="C4:C12" si="0">A4</f>
         <v>4</v>
       </c>
       <c r="D4">
-        <f>CEILING(B4/8,1)</f>
+        <f t="shared" ref="D4:D12" si="1">CEILING(B4/8,1)</f>
         <v>1</v>
       </c>
       <c r="E4">
-        <f>C4*D4</f>
+        <f t="shared" ref="E4:E12" si="2">C4*D4</f>
         <v>4</v>
       </c>
       <c r="F4">
-        <f>SUM(C4:E4)</f>
+        <f t="shared" ref="F4:F12" si="3">SUM(C4:E4)</f>
         <v>9</v>
       </c>
     </row>
@@ -1430,19 +1430,19 @@
         <v>16</v>
       </c>
       <c r="C5">
-        <f>A5</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="D5">
-        <f>CEILING(B5/8,1)</f>
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
       <c r="E5">
-        <f>C5*D5</f>
+        <f t="shared" si="2"/>
         <v>8</v>
       </c>
       <c r="F5">
-        <f>SUM(C5:E5)</f>
+        <f t="shared" si="3"/>
         <v>14</v>
       </c>
     </row>
@@ -1454,115 +1454,115 @@
         <v>24</v>
       </c>
       <c r="C6">
-        <f>A6</f>
+        <f t="shared" si="0"/>
         <v>4</v>
       </c>
       <c r="D6">
-        <f>CEILING(B6/8,1)</f>
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
       <c r="E6">
-        <f>C6*D6</f>
+        <f t="shared" si="2"/>
         <v>12</v>
       </c>
       <c r="F6">
-        <f>SUM(C6:E6)</f>
+        <f t="shared" si="3"/>
         <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" s="5">
-        <v>4</v>
-      </c>
-      <c r="B7" s="5">
+      <c r="A7" s="4">
+        <v>4</v>
+      </c>
+      <c r="B7" s="4">
         <v>32</v>
       </c>
-      <c r="C7" s="5">
-        <f>A7</f>
-        <v>4</v>
-      </c>
-      <c r="D7" s="5">
-        <f>CEILING(B7/8,1)</f>
-        <v>4</v>
-      </c>
-      <c r="E7" s="5">
-        <f>C7*D7</f>
+      <c r="C7" s="4">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="D7" s="4">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="E7" s="4">
+        <f t="shared" si="2"/>
         <v>16</v>
       </c>
-      <c r="F7" s="5">
-        <f>SUM(C7:E7)</f>
+      <c r="F7" s="4">
+        <f t="shared" si="3"/>
         <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="6">
+      <c r="A8" s="5">
         <v>8</v>
       </c>
-      <c r="B8" s="6">
+      <c r="B8" s="5">
         <v>8</v>
       </c>
-      <c r="C8" s="6">
-        <f>A8</f>
+      <c r="C8" s="5">
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="D8" s="6">
-        <f>CEILING(B8/8,1)</f>
+      <c r="D8" s="5">
+        <f t="shared" si="1"/>
         <v>1</v>
       </c>
-      <c r="E8" s="6">
-        <f>C8*D8</f>
+      <c r="E8" s="5">
+        <f t="shared" si="2"/>
         <v>8</v>
       </c>
-      <c r="F8" s="6">
-        <f>SUM(C8:E8)</f>
+      <c r="F8" s="5">
+        <f t="shared" si="3"/>
         <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="4">
+      <c r="A9" s="6">
         <v>8</v>
       </c>
-      <c r="B9" s="4">
+      <c r="B9" s="6">
         <v>16</v>
       </c>
-      <c r="C9" s="4">
-        <f>A9</f>
+      <c r="C9" s="6">
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="D9" s="4">
-        <f>CEILING(B9/8,1)</f>
+      <c r="D9" s="6">
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
-      <c r="E9" s="4">
-        <f>C9*D9</f>
+      <c r="E9" s="6">
+        <f t="shared" si="2"/>
         <v>16</v>
       </c>
-      <c r="F9" s="4">
-        <f>SUM(C9:E9)</f>
+      <c r="F9" s="6">
+        <f t="shared" si="3"/>
         <v>26</v>
       </c>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="7">
+      <c r="A10" s="6">
         <v>8</v>
       </c>
-      <c r="B10" s="5">
+      <c r="B10" s="7">
         <v>24</v>
       </c>
-      <c r="C10" s="5">
-        <f>A10</f>
+      <c r="C10" s="7">
+        <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="D10" s="5">
-        <f>CEILING(B10/8,1)</f>
+      <c r="D10" s="7">
+        <f t="shared" si="1"/>
         <v>3</v>
       </c>
-      <c r="E10" s="5">
-        <f>C10*D10</f>
+      <c r="E10" s="7">
+        <f t="shared" si="2"/>
         <v>24</v>
       </c>
-      <c r="F10" s="5">
-        <f>SUM(C10:E10)</f>
+      <c r="F10" s="7">
+        <f t="shared" si="3"/>
         <v>35</v>
       </c>
     </row>
@@ -1574,19 +1574,19 @@
         <v>16</v>
       </c>
       <c r="C11">
-        <f>A11</f>
+        <f t="shared" si="0"/>
         <v>9</v>
       </c>
       <c r="D11">
-        <f>CEILING(B11/8,1)</f>
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
       <c r="E11">
-        <f>C11*D11</f>
+        <f t="shared" si="2"/>
         <v>18</v>
       </c>
       <c r="F11">
-        <f>SUM(C11:E11)</f>
+        <f t="shared" si="3"/>
         <v>29</v>
       </c>
     </row>
@@ -1598,19 +1598,19 @@
         <v>16</v>
       </c>
       <c r="C12">
-        <f>A12</f>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="D12">
-        <f>CEILING(B12/8,1)</f>
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
       <c r="E12">
-        <f>C12*D12</f>
+        <f t="shared" si="2"/>
         <v>20</v>
       </c>
       <c r="F12">
-        <f>SUM(C12:E12)</f>
+        <f t="shared" si="3"/>
         <v>32</v>
       </c>
     </row>
@@ -1635,7 +1635,7 @@
     <col min="7" max="7" width="7.66666666666667" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:6">
+    <row r="1" spans="1:7">
       <c r="B1" s="1" t="s">
         <v>9</v>
       </c>

</xml_diff>